<commit_message>
Update puzzle answer spreadsheet
</commit_message>
<xml_diff>
--- a/02_寶箱密碼與生肖算式/言辵米角刀牛_13組生肖算式.xlsx
+++ b/02_寶箱密碼與生肖算式/言辵米角刀牛_13組生肖算式.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Easy's AI 製作資料夾\言辵米角刀牛\07_寶箱密碼與生肖算式\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Easy's AI 製作資料夾\言辵米角刀牛\02_寶箱密碼與生肖算式\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA87BD44-9DED-4C4B-A416-72868FF169EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F2BA71-D2AA-489B-9C28-945225F709A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="教師答案表" sheetId="1" r:id="rId1"/>
     <sheet name="學生題目表" sheetId="2" r:id="rId2"/>
     <sheet name="生肖對照與規則" sheetId="3" r:id="rId3"/>
+    <sheet name="鎖學生ipad白名單" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="143">
   <si>
     <t>言辵米・角刀牛｜13組生肖算式</t>
   </si>
@@ -451,6 +452,21 @@
   <si>
     <t>https://view.genially.com/68763e42ab77cefe054c0070</t>
     <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://easyshih-ux.github.io/puzzle-2026/01_解謎網站/開頭製作/index.html</t>
+  </si>
+  <si>
+    <t>https://easyshih-ux.github.io/puzzle-2026/01_解謎網站/開頭製作/index01.html</t>
+  </si>
+  <si>
+    <t>https://easyshih-ux.github.io/puzzle-2026/01_解謎網站/03首頁/home.html</t>
+  </si>
+  <si>
+    <t>https://easyshih-ux.github.io/puzzle-2026/01_解謎網站/03首頁/index_single_fixed.html</t>
+  </si>
+  <si>
+    <t>https://easyshih-ux.github.io/puzzle-2026/01_解謎網站/</t>
   </si>
 </sst>
 </file>
@@ -460,7 +476,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="000"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -566,6 +582,11 @@
       <color theme="10"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -654,7 +675,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -695,27 +716,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -949,36 +971,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="38" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
     </row>
     <row r="2" spans="1:13" ht="26" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
     </row>
     <row r="4" spans="1:13" ht="38" customHeight="1" thickBot="1">
       <c r="A4" s="1" t="s">
@@ -1059,7 +1081,7 @@
         <f t="shared" ref="L5:L17" si="0">C5+E5+G5+I5+K5</f>
         <v>440</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="M5" s="14" t="s">
         <v>137</v>
       </c>
     </row>
@@ -1590,24 +1612,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="38" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="2" spans="1:6" ht="26" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="4" spans="1:6" ht="48" customHeight="1">
       <c r="A4" s="6" t="s">
@@ -1911,28 +1933,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="38" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
     </row>
     <row r="2" spans="1:8" ht="26" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
     </row>
     <row r="4" spans="1:8" ht="26" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -1941,13 +1963,13 @@
       <c r="B4" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
     </row>
     <row r="5" spans="1:8" ht="28.05" customHeight="1">
       <c r="A5" s="11" t="s">
@@ -1956,13 +1978,13 @@
       <c r="B5" s="10">
         <v>1</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" ht="28.05" customHeight="1">
       <c r="A6" s="11" t="s">
@@ -1971,13 +1993,13 @@
       <c r="B6" s="10">
         <v>2</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
     </row>
     <row r="7" spans="1:8" ht="28.05" customHeight="1">
       <c r="A7" s="11" t="s">
@@ -1986,13 +2008,13 @@
       <c r="B7" s="10">
         <v>3</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
     </row>
     <row r="8" spans="1:8" ht="28.05" customHeight="1">
       <c r="A8" s="11" t="s">
@@ -2001,13 +2023,13 @@
       <c r="B8" s="10">
         <v>4</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
     </row>
     <row r="9" spans="1:8" ht="28.05" customHeight="1">
       <c r="A9" s="11" t="s">
@@ -2016,13 +2038,13 @@
       <c r="B9" s="10">
         <v>5</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
     </row>
     <row r="10" spans="1:8" ht="28.05" customHeight="1">
       <c r="A10" s="11" t="s">
@@ -2031,13 +2053,13 @@
       <c r="B10" s="10">
         <v>6</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
     </row>
     <row r="11" spans="1:8" ht="26" customHeight="1">
       <c r="A11" s="11" t="s">
@@ -2054,13 +2076,13 @@
       <c r="B12" s="10">
         <v>8</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
     </row>
     <row r="13" spans="1:8" ht="32" customHeight="1">
       <c r="A13" s="11" t="s">
@@ -2069,13 +2091,13 @@
       <c r="B13" s="10">
         <v>9</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
     </row>
     <row r="14" spans="1:8" ht="32" customHeight="1">
       <c r="A14" s="11" t="s">
@@ -2084,13 +2106,13 @@
       <c r="B14" s="10">
         <v>10</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
     </row>
     <row r="15" spans="1:8" ht="32" customHeight="1">
       <c r="A15" s="11" t="s">
@@ -2099,13 +2121,13 @@
       <c r="B15" s="10">
         <v>11</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
     </row>
     <row r="16" spans="1:8" ht="26" customHeight="1">
       <c r="A16" s="11" t="s">
@@ -2117,11 +2139,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="D15:H15"/>
@@ -2130,8 +2147,120 @@
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D12:H12"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F2E15CA-0336-430D-8EC2-C619EDAC25C0}">
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
+  <cols>
+    <col min="1" max="1" width="66.4375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="21" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="21" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="21" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="21" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="14" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="12" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="12" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="12" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="12" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="12" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="13" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A6" r:id="rId1" xr:uid="{BAC31A04-9B37-41E8-858B-75F296FA2A45}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>